<commit_message>
Simplify video workflows and add observability
</commit_message>
<xml_diff>
--- a/app/static/templates/digital_human-batch-template.xlsx
+++ b/app/static/templates/digital_human-batch-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="批量任务" sheetId="1" r:id="R29b76c61dd854e2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="2" r:id="Rc9c88a90be214bba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="批量任务" sheetId="1" r:id="Rcdaaeacf8e054a72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="2" r:id="R608fbed42dd54fa8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -44,20 +44,12 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="7">
+  <x:borders count="6">
     <x:border/>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FF0E4A98"/>
       </x:left>
-      <x:top style="thin">
-        <x:color rgb="FF0E4A98"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FF0E4A98"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
       <x:top style="thin">
         <x:color rgb="FF0E4A98"/>
       </x:top>
@@ -98,38 +90,43 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="18">
+  <x:cellXfs count="19">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -333,56 +330,25 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="42" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="80" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="6" t="str">
+      <x:c r="A1" s="5" t="str">
         <x:v>任务编号</x:v>
       </x:c>
-      <x:c r="B1" s="7" t="str">
-        <x:v>图片文件</x:v>
-      </x:c>
-      <x:c r="C1" s="7" t="str">
-        <x:v>总参考音频（上传模式填写）</x:v>
-      </x:c>
-      <x:c r="D1" s="7" t="str">
-        <x:v>口播脚本（语音生成模式填写）</x:v>
-      </x:c>
-      <x:c r="E1" s="7" t="str">
+      <x:c r="B1" s="6" t="str">
         <x:v>提示词</x:v>
       </x:c>
-      <x:c r="F1" s="7" t="str">
-        <x:v>左人物音频</x:v>
-      </x:c>
-      <x:c r="G1" s="8" t="str">
-        <x:v>右人物音频</x:v>
-      </x:c>
     </x:row>
     <x:row r="2" ht="46" customHeight="1">
-      <x:c r="A2" s="11" t="str">
+      <x:c r="A2" s="9" t="str">
         <x:v>TASK-001</x:v>
       </x:c>
-      <x:c r="B2" s="11" t="str">
-        <x:v>person-001.png</x:v>
-      </x:c>
-      <x:c r="C2" s="11" t="str">
-        <x:v>voice-001.mp3</x:v>
-      </x:c>
-      <x:c r="D2" s="11" t="str">
-        <x:v>今天给大家介绍这款产品。</x:v>
-      </x:c>
-      <x:c r="E2" s="11" t="str">
+      <x:c r="B2" s="9" t="str">
         <x:v>人物自然地说话，镜头保持稳定。</x:v>
       </x:c>
-      <x:c r="F2" s="11" t="str"/>
-      <x:c r="G2" s="11" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -393,40 +359,40 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="72" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>适用模式</x:v>
+        <x:v>项目</x:v>
       </x:c>
       <x:c r="B1" s="2" t="str">
         <x:v>说明</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="15" t="str">
-        <x:v>上传音频</x:v>
-      </x:c>
-      <x:c r="B2" s="15" t="str">
-        <x:v>填写图片文件、总参考音频和提示词；口播脚本可以留空。</x:v>
+      <x:c r="A2" s="16" t="str">
+        <x:v>表格内容</x:v>
+      </x:c>
+      <x:c r="B2" s="13" t="str">
+        <x:v>只填写任务编号和提示词，不填写任何图片或音频文件名。</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="16" t="str">
-        <x:v>脚本生成语音</x:v>
-      </x:c>
-      <x:c r="B3" s="16" t="str">
-        <x:v>填写图片文件、口播脚本和提示词；总参考音频留空。只支持单人模式。</x:v>
+      <x:c r="A3" s="17" t="str">
+        <x:v>素材对应</x:v>
+      </x:c>
+      <x:c r="B3" s="14" t="str">
+        <x:v>图片和总参考音频在网页分开上传；各自第 1、2、3……项对应表格第 1、2、3……行。</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="17" t="str">
-        <x:v>文件匹配</x:v>
-      </x:c>
-      <x:c r="B4" s="17" t="str">
-        <x:v>文件名必须包含扩展名，并与上传文件的完整名称一致。</x:v>
+      <x:c r="A4" s="18" t="str">
+        <x:v>双人模式</x:v>
+      </x:c>
+      <x:c r="B4" s="15" t="str">
+        <x:v>左人物音频、右人物音频也分别上传，并按各自序号对应同一行。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>